<commit_message>
Added new RDF data schemes and visual schemes for education-table18-19, fixed XLSX spreadsheets for education-table18-19
</commit_message>
<xml_diff>
--- a/sources/table_normalization/xlsx/education-table18.xlsx
+++ b/sources/table_normalization/xlsx/education-table18.xlsx
@@ -187,8 +187,8 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <numFmts count="2">
-    <numFmt numFmtId="168" formatCode="#,##0_)"/>
-    <numFmt numFmtId="169" formatCode="#,##0.0_)"/>
+    <numFmt numFmtId="164" formatCode="#,##0_)"/>
+    <numFmt numFmtId="165" formatCode="#,##0.0_)"/>
   </numFmts>
   <fonts count="17">
     <font>
@@ -833,7 +833,7 @@
     <xf numFmtId="0" fontId="15" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="15" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="146">
+  <cellXfs count="142">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="2" applyFont="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="2" applyFont="1" applyAlignment="1">
@@ -860,159 +860,159 @@
     <xf numFmtId="0" fontId="3" fillId="2" borderId="9" xfId="3" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="168" fontId="3" fillId="2" borderId="4" xfId="2" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right"/>
-    </xf>
-    <xf numFmtId="169" fontId="3" fillId="2" borderId="0" xfId="2" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="164" fontId="3" fillId="2" borderId="4" xfId="2" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="165" fontId="3" fillId="2" borderId="0" xfId="2" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="10" xfId="5" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="11" xfId="5" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="168" fontId="3" fillId="0" borderId="12" xfId="2" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right"/>
-    </xf>
-    <xf numFmtId="169" fontId="3" fillId="0" borderId="13" xfId="2" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="164" fontId="3" fillId="0" borderId="12" xfId="2" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="165" fontId="3" fillId="0" borderId="13" xfId="2" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="2" borderId="14" xfId="5" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="2" borderId="14" xfId="5" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="168" fontId="3" fillId="2" borderId="6" xfId="2" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right"/>
-    </xf>
-    <xf numFmtId="169" fontId="3" fillId="2" borderId="15" xfId="2" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="164" fontId="3" fillId="2" borderId="6" xfId="2" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="165" fontId="3" fillId="2" borderId="15" xfId="2" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="10" xfId="5" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="168" fontId="3" fillId="0" borderId="16" xfId="2" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right"/>
-    </xf>
-    <xf numFmtId="169" fontId="3" fillId="0" borderId="0" xfId="2" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="164" fontId="3" fillId="0" borderId="16" xfId="2" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="165" fontId="3" fillId="0" borderId="0" xfId="2" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="2" borderId="10" xfId="5" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="2" borderId="11" xfId="5" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="168" fontId="3" fillId="2" borderId="12" xfId="2" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right"/>
-    </xf>
-    <xf numFmtId="169" fontId="3" fillId="2" borderId="13" xfId="2" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="164" fontId="3" fillId="2" borderId="12" xfId="2" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="165" fontId="3" fillId="2" borderId="13" xfId="2" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="14" xfId="5" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="14" xfId="5" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="168" fontId="3" fillId="0" borderId="6" xfId="2" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right"/>
-    </xf>
-    <xf numFmtId="169" fontId="3" fillId="0" borderId="15" xfId="2" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="164" fontId="3" fillId="0" borderId="6" xfId="2" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="165" fontId="3" fillId="0" borderId="15" xfId="2" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="2" borderId="10" xfId="5" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="168" fontId="3" fillId="2" borderId="16" xfId="2" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="164" fontId="3" fillId="2" borderId="16" xfId="2" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
     <xf numFmtId="0" fontId="10" fillId="2" borderId="17" xfId="5" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="2" borderId="17" xfId="5" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="168" fontId="3" fillId="2" borderId="18" xfId="2" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right"/>
-    </xf>
-    <xf numFmtId="169" fontId="3" fillId="2" borderId="1" xfId="2" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="164" fontId="3" fillId="2" borderId="18" xfId="2" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="165" fontId="3" fillId="2" borderId="1" xfId="2" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
     <xf numFmtId="0" fontId="11" fillId="0" borderId="0" xfId="2" applyFont="1"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="2" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="2" applyFont="1" applyFill="1"/>
-    <xf numFmtId="169" fontId="3" fillId="2" borderId="25" xfId="2" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right"/>
-    </xf>
-    <xf numFmtId="168" fontId="3" fillId="2" borderId="0" xfId="2" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right"/>
-    </xf>
-    <xf numFmtId="169" fontId="3" fillId="0" borderId="26" xfId="2" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right"/>
-    </xf>
-    <xf numFmtId="168" fontId="3" fillId="0" borderId="13" xfId="2" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right"/>
-    </xf>
-    <xf numFmtId="169" fontId="3" fillId="2" borderId="27" xfId="2" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right"/>
-    </xf>
-    <xf numFmtId="168" fontId="3" fillId="2" borderId="15" xfId="2" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right"/>
-    </xf>
-    <xf numFmtId="169" fontId="3" fillId="0" borderId="25" xfId="2" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right"/>
-    </xf>
-    <xf numFmtId="168" fontId="3" fillId="0" borderId="0" xfId="2" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right"/>
-    </xf>
-    <xf numFmtId="169" fontId="3" fillId="2" borderId="26" xfId="2" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right"/>
-    </xf>
-    <xf numFmtId="168" fontId="3" fillId="2" borderId="13" xfId="2" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right"/>
-    </xf>
-    <xf numFmtId="169" fontId="3" fillId="0" borderId="27" xfId="2" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right"/>
-    </xf>
-    <xf numFmtId="168" fontId="3" fillId="0" borderId="15" xfId="2" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right"/>
-    </xf>
-    <xf numFmtId="169" fontId="3" fillId="2" borderId="28" xfId="2" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right"/>
-    </xf>
-    <xf numFmtId="168" fontId="3" fillId="2" borderId="1" xfId="2" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="165" fontId="3" fillId="2" borderId="25" xfId="2" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="164" fontId="3" fillId="2" borderId="0" xfId="2" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="165" fontId="3" fillId="0" borderId="26" xfId="2" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="164" fontId="3" fillId="0" borderId="13" xfId="2" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="165" fontId="3" fillId="2" borderId="27" xfId="2" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="164" fontId="3" fillId="2" borderId="15" xfId="2" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="165" fontId="3" fillId="0" borderId="25" xfId="2" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="164" fontId="3" fillId="0" borderId="0" xfId="2" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="165" fontId="3" fillId="2" borderId="26" xfId="2" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="164" fontId="3" fillId="2" borderId="13" xfId="2" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="165" fontId="3" fillId="0" borderId="27" xfId="2" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="164" fontId="3" fillId="0" borderId="15" xfId="2" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="165" fontId="3" fillId="2" borderId="28" xfId="2" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="164" fontId="3" fillId="2" borderId="1" xfId="2" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
     <xf numFmtId="0" fontId="12" fillId="3" borderId="0" xfId="2" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="168" fontId="3" fillId="2" borderId="33" xfId="2" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right"/>
-    </xf>
-    <xf numFmtId="169" fontId="3" fillId="2" borderId="5" xfId="2" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right"/>
-    </xf>
-    <xf numFmtId="168" fontId="3" fillId="0" borderId="34" xfId="2" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right"/>
-    </xf>
-    <xf numFmtId="169" fontId="3" fillId="0" borderId="35" xfId="2" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right"/>
-    </xf>
-    <xf numFmtId="168" fontId="3" fillId="2" borderId="36" xfId="2" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right"/>
-    </xf>
-    <xf numFmtId="169" fontId="3" fillId="2" borderId="7" xfId="2" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right"/>
-    </xf>
-    <xf numFmtId="168" fontId="3" fillId="0" borderId="33" xfId="2" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right"/>
-    </xf>
-    <xf numFmtId="169" fontId="3" fillId="0" borderId="5" xfId="2" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right"/>
-    </xf>
-    <xf numFmtId="168" fontId="3" fillId="2" borderId="34" xfId="2" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right"/>
-    </xf>
-    <xf numFmtId="169" fontId="3" fillId="2" borderId="35" xfId="2" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right"/>
-    </xf>
-    <xf numFmtId="168" fontId="3" fillId="0" borderId="36" xfId="2" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right"/>
-    </xf>
-    <xf numFmtId="169" fontId="3" fillId="0" borderId="7" xfId="2" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right"/>
-    </xf>
-    <xf numFmtId="168" fontId="3" fillId="2" borderId="37" xfId="2" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right"/>
-    </xf>
-    <xf numFmtId="169" fontId="3" fillId="2" borderId="8" xfId="2" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="164" fontId="3" fillId="2" borderId="33" xfId="2" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="165" fontId="3" fillId="2" borderId="5" xfId="2" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="164" fontId="3" fillId="0" borderId="34" xfId="2" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="165" fontId="3" fillId="0" borderId="35" xfId="2" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="164" fontId="3" fillId="2" borderId="36" xfId="2" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="165" fontId="3" fillId="2" borderId="7" xfId="2" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="164" fontId="3" fillId="0" borderId="33" xfId="2" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="165" fontId="3" fillId="0" borderId="5" xfId="2" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="164" fontId="3" fillId="2" borderId="34" xfId="2" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="165" fontId="3" fillId="2" borderId="35" xfId="2" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="164" fontId="3" fillId="0" borderId="36" xfId="2" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="165" fontId="3" fillId="0" borderId="7" xfId="2" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="164" fontId="3" fillId="2" borderId="37" xfId="2" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="165" fontId="3" fillId="2" borderId="8" xfId="2" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
     <xf numFmtId="1" fontId="6" fillId="0" borderId="0" xfId="4" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
@@ -1020,70 +1020,107 @@
     </xf>
     <xf numFmtId="0" fontId="11" fillId="0" borderId="0" xfId="2" applyFont="1" applyBorder="1"/>
     <xf numFmtId="37" fontId="3" fillId="2" borderId="40" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="169" fontId="3" fillId="2" borderId="33" xfId="2" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="165" fontId="3" fillId="2" borderId="33" xfId="2" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="37" fontId="3" fillId="0" borderId="42" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="169" fontId="3" fillId="0" borderId="34" xfId="2" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="165" fontId="3" fillId="0" borderId="34" xfId="2" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="37" fontId="3" fillId="2" borderId="43" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="169" fontId="3" fillId="2" borderId="36" xfId="2" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="165" fontId="3" fillId="2" borderId="36" xfId="2" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="37" fontId="3" fillId="0" borderId="40" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="169" fontId="3" fillId="0" borderId="33" xfId="2" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="165" fontId="3" fillId="0" borderId="33" xfId="2" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="37" fontId="3" fillId="2" borderId="42" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="169" fontId="3" fillId="2" borderId="34" xfId="2" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="165" fontId="3" fillId="2" borderId="34" xfId="2" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="37" fontId="3" fillId="0" borderId="43" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="169" fontId="3" fillId="0" borderId="36" xfId="2" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="165" fontId="3" fillId="0" borderId="36" xfId="2" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="37" fontId="3" fillId="2" borderId="41" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="169" fontId="3" fillId="2" borderId="37" xfId="2" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="165" fontId="3" fillId="2" borderId="37" xfId="2" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="1" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="168" fontId="3" fillId="2" borderId="0" xfId="2" quotePrefix="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right"/>
-    </xf>
-    <xf numFmtId="168" fontId="3" fillId="0" borderId="12" xfId="2" quotePrefix="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right"/>
-    </xf>
-    <xf numFmtId="168" fontId="3" fillId="0" borderId="13" xfId="2" quotePrefix="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right"/>
-    </xf>
-    <xf numFmtId="168" fontId="3" fillId="2" borderId="13" xfId="2" quotePrefix="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right"/>
-    </xf>
-    <xf numFmtId="168" fontId="3" fillId="2" borderId="12" xfId="2" quotePrefix="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right"/>
-    </xf>
-    <xf numFmtId="168" fontId="3" fillId="0" borderId="15" xfId="2" quotePrefix="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right"/>
-    </xf>
-    <xf numFmtId="168" fontId="3" fillId="2" borderId="16" xfId="2" quotePrefix="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right"/>
-    </xf>
-    <xf numFmtId="168" fontId="3" fillId="2" borderId="15" xfId="2" quotePrefix="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right"/>
-    </xf>
-    <xf numFmtId="168" fontId="3" fillId="2" borderId="6" xfId="2" quotePrefix="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right"/>
-    </xf>
-    <xf numFmtId="168" fontId="3" fillId="0" borderId="16" xfId="2" quotePrefix="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right"/>
-    </xf>
-    <xf numFmtId="168" fontId="3" fillId="0" borderId="0" xfId="2" quotePrefix="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right"/>
-    </xf>
-    <xf numFmtId="168" fontId="3" fillId="0" borderId="33" xfId="2" quotePrefix="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right"/>
-    </xf>
-    <xf numFmtId="168" fontId="3" fillId="2" borderId="33" xfId="2" quotePrefix="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right"/>
-    </xf>
-    <xf numFmtId="168" fontId="3" fillId="0" borderId="34" xfId="2" quotePrefix="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right"/>
-    </xf>
-    <xf numFmtId="168" fontId="3" fillId="2" borderId="34" xfId="2" quotePrefix="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right"/>
-    </xf>
-    <xf numFmtId="168" fontId="3" fillId="0" borderId="6" xfId="2" quotePrefix="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right"/>
-    </xf>
-    <xf numFmtId="168" fontId="3" fillId="2" borderId="1" xfId="2" quotePrefix="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right"/>
+    <xf numFmtId="164" fontId="3" fillId="2" borderId="0" xfId="2" quotePrefix="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="164" fontId="3" fillId="0" borderId="12" xfId="2" quotePrefix="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="164" fontId="3" fillId="0" borderId="13" xfId="2" quotePrefix="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="164" fontId="3" fillId="2" borderId="13" xfId="2" quotePrefix="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="164" fontId="3" fillId="2" borderId="12" xfId="2" quotePrefix="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="164" fontId="3" fillId="0" borderId="15" xfId="2" quotePrefix="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="164" fontId="3" fillId="2" borderId="16" xfId="2" quotePrefix="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="164" fontId="3" fillId="2" borderId="15" xfId="2" quotePrefix="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="164" fontId="3" fillId="2" borderId="6" xfId="2" quotePrefix="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="164" fontId="3" fillId="0" borderId="16" xfId="2" quotePrefix="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="164" fontId="3" fillId="0" borderId="0" xfId="2" quotePrefix="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="164" fontId="3" fillId="0" borderId="33" xfId="2" quotePrefix="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="164" fontId="3" fillId="2" borderId="33" xfId="2" quotePrefix="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="164" fontId="3" fillId="0" borderId="34" xfId="2" quotePrefix="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="164" fontId="3" fillId="2" borderId="34" xfId="2" quotePrefix="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="164" fontId="3" fillId="0" borderId="6" xfId="2" quotePrefix="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="164" fontId="3" fillId="2" borderId="1" xfId="2" quotePrefix="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="1" fontId="9" fillId="5" borderId="1" xfId="3" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" wrapText="1"/>
+    </xf>
+    <xf numFmtId="1" fontId="9" fillId="5" borderId="8" xfId="3" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" wrapText="1"/>
+    </xf>
+    <xf numFmtId="1" fontId="9" fillId="5" borderId="18" xfId="3" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" wrapText="1"/>
+    </xf>
+    <xf numFmtId="1" fontId="9" fillId="5" borderId="24" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" wrapText="1"/>
+    </xf>
+    <xf numFmtId="1" fontId="9" fillId="5" borderId="32" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="4" borderId="0" xfId="2" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="4" borderId="0" xfId="2" quotePrefix="1" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="4" borderId="0" xfId="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="1" fontId="9" fillId="0" borderId="4" xfId="3" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="1" fontId="9" fillId="0" borderId="3" xfId="3" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="1" fontId="9" fillId="0" borderId="6" xfId="3" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="1" fontId="9" fillId="0" borderId="7" xfId="3" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="37" fontId="7" fillId="4" borderId="0" xfId="5" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left" wrapText="1"/>
     </xf>
     <xf numFmtId="1" fontId="9" fillId="0" borderId="21" xfId="3" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" wrapText="1"/>
@@ -1100,98 +1137,49 @@
     <xf numFmtId="1" fontId="9" fillId="0" borderId="31" xfId="3" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="1" fontId="9" fillId="0" borderId="4" xfId="3" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="1" fontId="9" fillId="0" borderId="3" xfId="3" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="1" fontId="9" fillId="0" borderId="6" xfId="3" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="1" fontId="9" fillId="0" borderId="7" xfId="3" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="37" fontId="7" fillId="4" borderId="0" xfId="5" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="left" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="9" fillId="5" borderId="2" xfId="3" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="9" fillId="5" borderId="0" xfId="3" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="5" borderId="1" xfId="3" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="9" fillId="5" borderId="3" xfId="3" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="9" fillId="5" borderId="0" xfId="3" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="9" fillId="5" borderId="5" xfId="3" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="9" fillId="5" borderId="1" xfId="3" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="9" fillId="5" borderId="8" xfId="3" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="1" fontId="9" fillId="5" borderId="4" xfId="3" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="1" fontId="9" fillId="5" borderId="3" xfId="3" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="1" fontId="9" fillId="5" borderId="6" xfId="3" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="1" fontId="9" fillId="5" borderId="7" xfId="3" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="1" fontId="9" fillId="5" borderId="1" xfId="3" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" wrapText="1"/>
-    </xf>
-    <xf numFmtId="1" fontId="9" fillId="5" borderId="8" xfId="3" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" wrapText="1"/>
-    </xf>
-    <xf numFmtId="1" fontId="9" fillId="5" borderId="18" xfId="3" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" wrapText="1"/>
-    </xf>
-    <xf numFmtId="1" fontId="9" fillId="5" borderId="24" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" wrapText="1"/>
-    </xf>
-    <xf numFmtId="1" fontId="9" fillId="5" borderId="32" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" wrapText="1"/>
-    </xf>
     <xf numFmtId="1" fontId="9" fillId="5" borderId="38" xfId="3" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="1" fontId="9" fillId="5" borderId="40" xfId="3" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="1" fontId="9" fillId="5" borderId="41" xfId="3" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="1" fontId="9" fillId="5" borderId="39" xfId="3" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="1" fontId="9" fillId="5" borderId="40" xfId="3" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="1" fontId="9" fillId="5" borderId="33" xfId="3" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="1" fontId="9" fillId="5" borderId="41" xfId="3" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="1" fontId="9" fillId="5" borderId="37" xfId="3" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="4" borderId="0" xfId="2" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="4" borderId="0" xfId="2" quotePrefix="1" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="4" borderId="0" xfId="1" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="1" fontId="9" fillId="5" borderId="19" xfId="3" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="1" fontId="9" fillId="0" borderId="19" xfId="3" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="1" fontId="9" fillId="5" borderId="20" xfId="3" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="1" fontId="9" fillId="0" borderId="20" xfId="3" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="1" fontId="9" fillId="5" borderId="30" xfId="3" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="1" fontId="9" fillId="0" borderId="30" xfId="3" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
@@ -1575,34 +1563,34 @@
       <c r="Z1" s="11"/>
     </row>
     <row r="2" spans="1:26" s="2" customFormat="1" ht="15" customHeight="1">
-      <c r="A2" s="118" t="s">
-        <v>0</v>
-      </c>
-      <c r="B2" s="118"/>
-      <c r="C2" s="118"/>
-      <c r="D2" s="118"/>
-      <c r="E2" s="118"/>
-      <c r="F2" s="118"/>
-      <c r="G2" s="118"/>
-      <c r="H2" s="118"/>
-      <c r="I2" s="118"/>
-      <c r="J2" s="118"/>
-      <c r="K2" s="118"/>
-      <c r="L2" s="118"/>
-      <c r="M2" s="118"/>
-      <c r="N2" s="118"/>
-      <c r="O2" s="118"/>
-      <c r="P2" s="118"/>
-      <c r="Q2" s="118"/>
-      <c r="R2" s="118"/>
-      <c r="S2" s="118"/>
-      <c r="T2" s="118"/>
-      <c r="U2" s="118"/>
-      <c r="V2" s="118"/>
-      <c r="W2" s="118"/>
-      <c r="X2" s="118"/>
-      <c r="Y2" s="118"/>
-      <c r="Z2" s="118"/>
+      <c r="A2" s="121" t="s">
+        <v>0</v>
+      </c>
+      <c r="B2" s="121"/>
+      <c r="C2" s="121"/>
+      <c r="D2" s="121"/>
+      <c r="E2" s="121"/>
+      <c r="F2" s="121"/>
+      <c r="G2" s="121"/>
+      <c r="H2" s="121"/>
+      <c r="I2" s="121"/>
+      <c r="J2" s="121"/>
+      <c r="K2" s="121"/>
+      <c r="L2" s="121"/>
+      <c r="M2" s="121"/>
+      <c r="N2" s="121"/>
+      <c r="O2" s="121"/>
+      <c r="P2" s="121"/>
+      <c r="Q2" s="121"/>
+      <c r="R2" s="121"/>
+      <c r="S2" s="121"/>
+      <c r="T2" s="121"/>
+      <c r="U2" s="121"/>
+      <c r="V2" s="121"/>
+      <c r="W2" s="121"/>
+      <c r="X2" s="121"/>
+      <c r="Y2" s="121"/>
+      <c r="Z2" s="121"/>
     </row>
     <row r="3" spans="1:26" s="1" customFormat="1" ht="15" customHeight="1">
       <c r="A3" s="12"/>
@@ -1633,164 +1621,164 @@
       <c r="Z3" s="13"/>
     </row>
     <row r="4" spans="1:26" s="3" customFormat="1" ht="25" customHeight="1">
-      <c r="A4" s="119" t="s">
+      <c r="A4" s="127" t="s">
         <v>1</v>
       </c>
-      <c r="B4" s="120" t="s">
+      <c r="B4" s="130" t="s">
         <v>2</v>
       </c>
-      <c r="C4" s="125" t="s">
+      <c r="C4" s="117" t="s">
         <v>3</v>
       </c>
-      <c r="D4" s="126"/>
-      <c r="E4" s="143" t="s">
+      <c r="D4" s="118"/>
+      <c r="E4" s="139" t="s">
         <v>4</v>
       </c>
-      <c r="F4" s="144"/>
-      <c r="G4" s="144"/>
-      <c r="H4" s="144"/>
-      <c r="I4" s="144"/>
-      <c r="J4" s="144"/>
-      <c r="K4" s="144"/>
-      <c r="L4" s="144"/>
-      <c r="M4" s="144"/>
-      <c r="N4" s="144"/>
-      <c r="O4" s="144"/>
-      <c r="P4" s="144"/>
-      <c r="Q4" s="144"/>
-      <c r="R4" s="145"/>
-      <c r="S4" s="114" t="s">
+      <c r="F4" s="140"/>
+      <c r="G4" s="140"/>
+      <c r="H4" s="140"/>
+      <c r="I4" s="140"/>
+      <c r="J4" s="140"/>
+      <c r="K4" s="140"/>
+      <c r="L4" s="140"/>
+      <c r="M4" s="140"/>
+      <c r="N4" s="140"/>
+      <c r="O4" s="140"/>
+      <c r="P4" s="140"/>
+      <c r="Q4" s="140"/>
+      <c r="R4" s="141"/>
+      <c r="S4" s="117" t="s">
         <v>5</v>
       </c>
-      <c r="T4" s="115"/>
-      <c r="U4" s="114" t="s">
+      <c r="T4" s="118"/>
+      <c r="U4" s="117" t="s">
         <v>6</v>
       </c>
-      <c r="V4" s="115"/>
-      <c r="W4" s="114" t="s">
+      <c r="V4" s="118"/>
+      <c r="W4" s="117" t="s">
         <v>7</v>
       </c>
-      <c r="X4" s="115"/>
-      <c r="Y4" s="134" t="s">
+      <c r="X4" s="118"/>
+      <c r="Y4" s="133" t="s">
         <v>8</v>
       </c>
-      <c r="Z4" s="135" t="s">
+      <c r="Z4" s="136" t="s">
         <v>9</v>
       </c>
     </row>
     <row r="5" spans="1:26" s="3" customFormat="1" ht="25" customHeight="1">
-      <c r="A5" s="121"/>
-      <c r="B5" s="122"/>
-      <c r="C5" s="127"/>
-      <c r="D5" s="128"/>
-      <c r="E5" s="109" t="s">
+      <c r="A5" s="128"/>
+      <c r="B5" s="131"/>
+      <c r="C5" s="119"/>
+      <c r="D5" s="120"/>
+      <c r="E5" s="122" t="s">
         <v>10</v>
       </c>
-      <c r="F5" s="110"/>
-      <c r="G5" s="111" t="s">
+      <c r="F5" s="123"/>
+      <c r="G5" s="124" t="s">
         <v>11</v>
       </c>
-      <c r="H5" s="110"/>
-      <c r="I5" s="112" t="s">
+      <c r="H5" s="123"/>
+      <c r="I5" s="125" t="s">
         <v>12</v>
       </c>
-      <c r="J5" s="110"/>
-      <c r="K5" s="112" t="s">
+      <c r="J5" s="123"/>
+      <c r="K5" s="125" t="s">
         <v>13</v>
       </c>
-      <c r="L5" s="110"/>
-      <c r="M5" s="112" t="s">
+      <c r="L5" s="123"/>
+      <c r="M5" s="125" t="s">
         <v>14</v>
       </c>
-      <c r="N5" s="110"/>
-      <c r="O5" s="112" t="s">
+      <c r="N5" s="123"/>
+      <c r="O5" s="125" t="s">
         <v>15</v>
       </c>
-      <c r="P5" s="110"/>
-      <c r="Q5" s="112" t="s">
+      <c r="P5" s="123"/>
+      <c r="Q5" s="125" t="s">
         <v>16</v>
       </c>
-      <c r="R5" s="113"/>
-      <c r="S5" s="116"/>
-      <c r="T5" s="117"/>
-      <c r="U5" s="116"/>
-      <c r="V5" s="117"/>
-      <c r="W5" s="116"/>
-      <c r="X5" s="117"/>
-      <c r="Y5" s="136"/>
+      <c r="R5" s="126"/>
+      <c r="S5" s="119"/>
+      <c r="T5" s="120"/>
+      <c r="U5" s="119"/>
+      <c r="V5" s="120"/>
+      <c r="W5" s="119"/>
+      <c r="X5" s="120"/>
+      <c r="Y5" s="134"/>
       <c r="Z5" s="137"/>
     </row>
     <row r="6" spans="1:26" s="3" customFormat="1" ht="15" customHeight="1">
-      <c r="A6" s="123"/>
-      <c r="B6" s="124"/>
-      <c r="C6" s="129" t="s">
+      <c r="A6" s="129"/>
+      <c r="B6" s="132"/>
+      <c r="C6" s="109" t="s">
         <v>17</v>
       </c>
-      <c r="D6" s="130" t="s">
+      <c r="D6" s="110" t="s">
         <v>18</v>
       </c>
-      <c r="E6" s="131" t="s">
+      <c r="E6" s="111" t="s">
         <v>17</v>
       </c>
-      <c r="F6" s="132" t="s">
+      <c r="F6" s="112" t="s">
         <v>19</v>
       </c>
-      <c r="G6" s="129" t="s">
+      <c r="G6" s="109" t="s">
         <v>17</v>
       </c>
-      <c r="H6" s="132" t="s">
+      <c r="H6" s="112" t="s">
         <v>19</v>
       </c>
-      <c r="I6" s="129" t="s">
+      <c r="I6" s="109" t="s">
         <v>17</v>
       </c>
-      <c r="J6" s="132" t="s">
+      <c r="J6" s="112" t="s">
         <v>19</v>
       </c>
-      <c r="K6" s="129" t="s">
+      <c r="K6" s="109" t="s">
         <v>17</v>
       </c>
-      <c r="L6" s="132" t="s">
+      <c r="L6" s="112" t="s">
         <v>19</v>
       </c>
-      <c r="M6" s="129" t="s">
+      <c r="M6" s="109" t="s">
         <v>17</v>
       </c>
-      <c r="N6" s="132" t="s">
+      <c r="N6" s="112" t="s">
         <v>19</v>
       </c>
-      <c r="O6" s="129" t="s">
+      <c r="O6" s="109" t="s">
         <v>17</v>
       </c>
-      <c r="P6" s="132" t="s">
+      <c r="P6" s="112" t="s">
         <v>19</v>
       </c>
-      <c r="Q6" s="129" t="s">
+      <c r="Q6" s="109" t="s">
         <v>17</v>
       </c>
-      <c r="R6" s="133" t="s">
+      <c r="R6" s="113" t="s">
         <v>19</v>
       </c>
-      <c r="S6" s="131" t="s">
+      <c r="S6" s="111" t="s">
         <v>17</v>
       </c>
-      <c r="T6" s="130" t="s">
+      <c r="T6" s="110" t="s">
         <v>18</v>
       </c>
-      <c r="U6" s="131" t="s">
+      <c r="U6" s="111" t="s">
         <v>17</v>
       </c>
-      <c r="V6" s="130" t="s">
+      <c r="V6" s="110" t="s">
         <v>18</v>
       </c>
-      <c r="W6" s="129" t="s">
+      <c r="W6" s="109" t="s">
         <v>17</v>
       </c>
-      <c r="X6" s="130" t="s">
+      <c r="X6" s="110" t="s">
         <v>18</v>
       </c>
-      <c r="Y6" s="138"/>
-      <c r="Z6" s="139"/>
+      <c r="Y6" s="135"/>
+      <c r="Z6" s="138"/>
     </row>
     <row r="7" spans="1:26" s="4" customFormat="1" ht="15" customHeight="1">
       <c r="A7" s="14"/>
@@ -4889,7 +4877,7 @@
       <c r="Z46" s="1"/>
     </row>
     <row r="47" spans="1:26" s="7" customFormat="1" ht="15" customHeight="1">
-      <c r="A47" s="140" t="str">
+      <c r="A47" s="114" t="str">
         <f>CONCATENATE("NOTE: Table reads:  Of all ",IF(ISTEXT(C9),LEFT(C9,3),TEXT(C9,"#,##0"))," public school students retained in kindergarten, ",IF(ISTEXT(E9),LEFT(E9,3),TEXT(E9,"#,##0"))," (",TEXT(F9,"0.0"),"%) were American Indian or Alaska Native, ",IF(ISTEXT(S9),LEFT(S9,3),TEXT(S9,"#,##0"))," (",TEXT(T9,"0.0"),"%) were students with disabilities served under the Individuals with Disabilities Education Act (IDEA), and ",IF(ISTEXT(U9),LEFT(U9,3),TEXT(U9,"#,##0"))," (",TEXT(V9,"0.0"),"%) were students with disabilities served solely under Section 504 of the Rehabilitation Act of 1973.")</f>
         <v>NOTE: Table reads:  Of all 2,560 public school students retained in kindergarten, 10 (0.4%) were American Indian or Alaska Native, 413 (16.1%) were students with disabilities served under the Individuals with Disabilities Education Act (IDEA), and 8 (0.3%) were students with disabilities served solely under Section 504 of the Rehabilitation Act of 1973.</v>
       </c>
@@ -4920,7 +4908,7 @@
       <c r="Z47" s="43"/>
     </row>
     <row r="48" spans="1:26" s="4" customFormat="1" ht="15" customHeight="1">
-      <c r="A48" s="141" t="s">
+      <c r="A48" s="115" t="s">
         <v>37</v>
       </c>
       <c r="B48" s="44"/>
@@ -4948,7 +4936,7 @@
       <c r="X48" s="45"/>
     </row>
     <row r="49" spans="1:26" s="7" customFormat="1" ht="14" customHeight="1">
-      <c r="A49" s="142" t="s">
+      <c r="A49" s="116" t="s">
         <v>38</v>
       </c>
       <c r="B49" s="5"/>
@@ -4979,6 +4967,7 @@
     </row>
   </sheetData>
   <mergeCells count="17">
+    <mergeCell ref="U4:V5"/>
     <mergeCell ref="W4:X5"/>
     <mergeCell ref="A2:Z2"/>
     <mergeCell ref="E4:R4"/>
@@ -4995,7 +4984,6 @@
     <mergeCell ref="Z4:Z6"/>
     <mergeCell ref="C4:D5"/>
     <mergeCell ref="S4:T5"/>
-    <mergeCell ref="U4:V5"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>